<commit_message>
Alteração na planilha Excell
</commit_message>
<xml_diff>
--- a/Arquivos-originais/Exercícios Práticos — Testes Manuais em Sites.xlsx
+++ b/Arquivos-originais/Exercícios Práticos — Testes Manuais em Sites.xlsx
@@ -5,19 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guga_\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a4d90896ecd236eb/Área de Trabalho/LumeStack/Development/Study/projetos/Arquivos-originais/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C72B51B-47C4-441C-9DFD-9E95468231D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{5C72B51B-47C4-441C-9DFD-9E95468231D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD4033FC-6F3F-476E-A8E2-ADD45B6856C8}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Caso de Teste" sheetId="1" r:id="rId1"/>
-    <sheet name="Bug Report - Caso 1" sheetId="2" r:id="rId2"/>
-    <sheet name="Relatório de Inconsistência - C" sheetId="3" r:id="rId3"/>
-    <sheet name="Lista de Erros Encontrados - Ca" sheetId="4" r:id="rId4"/>
-    <sheet name="Relatório comportamental espera" sheetId="5" r:id="rId5"/>
+    <sheet name="Bug Report" sheetId="2" r:id="rId2"/>
+    <sheet name="Relatório de Inconsistência" sheetId="3" r:id="rId3"/>
+    <sheet name="Lista de Erros Encontrados" sheetId="4" r:id="rId4"/>
+    <sheet name="Relatório comportamental" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -1282,18 +1282,6 @@
     <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1309,25 +1297,37 @@
     <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1897,7 +1897,7 @@
       <c r="E10" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="F10" s="38" t="s">
+      <c r="F10" s="32" t="s">
         <v>70</v>
       </c>
       <c r="G10" s="1"/>
@@ -1969,7 +1969,7 @@
       <c r="E12" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="F12" s="39" t="s">
+      <c r="F12" s="33" t="s">
         <v>53</v>
       </c>
       <c r="G12" s="1"/>
@@ -2009,7 +2009,7 @@
       <c r="E13" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="F13" s="38" t="s">
+      <c r="F13" s="32" t="s">
         <v>77</v>
       </c>
       <c r="G13" s="1"/>
@@ -2037,11 +2037,11 @@
       <c r="A14" s="11">
         <v>4</v>
       </c>
-      <c r="B14" s="32" t="s">
+      <c r="B14" s="43" t="s">
         <v>78</v>
       </c>
-      <c r="C14" s="33"/>
-      <c r="D14" s="33"/>
+      <c r="C14" s="44"/>
+      <c r="D14" s="44"/>
       <c r="E14" s="26"/>
       <c r="F14" s="26"/>
       <c r="G14" s="1"/>
@@ -2161,7 +2161,7 @@
       <c r="E17" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="F17" s="38" t="s">
+      <c r="F17" s="32" t="s">
         <v>107</v>
       </c>
       <c r="G17" s="1"/>
@@ -2201,7 +2201,7 @@
       <c r="E18" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="F18" s="38" t="s">
+      <c r="F18" s="32" t="s">
         <v>111</v>
       </c>
       <c r="G18" s="1"/>
@@ -2353,7 +2353,7 @@
       <c r="E22" s="21" t="s">
         <v>266</v>
       </c>
-      <c r="F22" s="38" t="s">
+      <c r="F22" s="32" t="s">
         <v>118</v>
       </c>
       <c r="G22" s="1"/>
@@ -2615,7 +2615,7 @@
       <c r="E30" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="F30" s="38" t="s">
+      <c r="F30" s="32" t="s">
         <v>127</v>
       </c>
       <c r="G30" s="30"/>
@@ -2655,7 +2655,7 @@
       <c r="E31" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="F31" s="38" t="s">
+      <c r="F31" s="32" t="s">
         <v>131</v>
       </c>
       <c r="G31" s="30"/>
@@ -2695,7 +2695,7 @@
       <c r="E32" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="F32" s="38" t="s">
+      <c r="F32" s="32" t="s">
         <v>136</v>
       </c>
       <c r="G32" s="30"/>
@@ -2735,7 +2735,7 @@
       <c r="E33" s="21" t="s">
         <v>140</v>
       </c>
-      <c r="F33" s="38" t="s">
+      <c r="F33" s="32" t="s">
         <v>141</v>
       </c>
       <c r="G33" s="30"/>
@@ -2775,7 +2775,7 @@
       <c r="E34" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="F34" s="38" t="s">
+      <c r="F34" s="32" t="s">
         <v>145</v>
       </c>
       <c r="G34" s="30"/>
@@ -2847,7 +2847,7 @@
       <c r="E36" s="21" t="s">
         <v>148</v>
       </c>
-      <c r="F36" s="38" t="s">
+      <c r="F36" s="32" t="s">
         <v>149</v>
       </c>
       <c r="G36" s="30"/>
@@ -2887,7 +2887,7 @@
       <c r="E37" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="F37" s="38" t="s">
+      <c r="F37" s="32" t="s">
         <v>152</v>
       </c>
       <c r="G37" s="30"/>
@@ -2927,7 +2927,7 @@
       <c r="E38" s="21" t="s">
         <v>271</v>
       </c>
-      <c r="F38" s="38" t="s">
+      <c r="F38" s="32" t="s">
         <v>155</v>
       </c>
       <c r="G38" s="30"/>
@@ -2999,7 +2999,7 @@
       <c r="E40" s="21" t="s">
         <v>159</v>
       </c>
-      <c r="F40" s="38" t="s">
+      <c r="F40" s="32" t="s">
         <v>160</v>
       </c>
       <c r="G40" s="1"/>
@@ -3039,7 +3039,7 @@
       <c r="E41" s="21" t="s">
         <v>163</v>
       </c>
-      <c r="F41" s="38" t="s">
+      <c r="F41" s="32" t="s">
         <v>164</v>
       </c>
       <c r="G41" s="1"/>
@@ -3079,7 +3079,7 @@
       <c r="E42" s="21" t="s">
         <v>168</v>
       </c>
-      <c r="F42" s="38" t="s">
+      <c r="F42" s="32" t="s">
         <v>169</v>
       </c>
       <c r="G42" s="1"/>
@@ -3119,7 +3119,7 @@
       <c r="E43" s="21" t="s">
         <v>173</v>
       </c>
-      <c r="F43" s="38" t="s">
+      <c r="F43" s="32" t="s">
         <v>174</v>
       </c>
       <c r="G43" s="1"/>
@@ -3191,7 +3191,7 @@
       <c r="E45" s="21" t="s">
         <v>272</v>
       </c>
-      <c r="F45" s="38" t="s">
+      <c r="F45" s="32" t="s">
         <v>177</v>
       </c>
       <c r="G45" s="1"/>
@@ -3231,7 +3231,7 @@
       <c r="E46" s="21" t="s">
         <v>273</v>
       </c>
-      <c r="F46" s="38" t="s">
+      <c r="F46" s="32" t="s">
         <v>179</v>
       </c>
       <c r="G46" s="1"/>
@@ -3493,7 +3493,7 @@
       <c r="E54" s="21" t="s">
         <v>261</v>
       </c>
-      <c r="F54" s="38" t="s">
+      <c r="F54" s="32" t="s">
         <v>187</v>
       </c>
       <c r="G54" s="1"/>
@@ -3565,7 +3565,7 @@
       <c r="E56" s="21" t="s">
         <v>261</v>
       </c>
-      <c r="F56" s="38" t="s">
+      <c r="F56" s="32" t="s">
         <v>187</v>
       </c>
       <c r="G56" s="1"/>
@@ -3605,7 +3605,7 @@
       <c r="E57" s="21" t="s">
         <v>276</v>
       </c>
-      <c r="F57" s="38" t="s">
+      <c r="F57" s="32" t="s">
         <v>192</v>
       </c>
       <c r="G57" s="1"/>
@@ -3677,7 +3677,7 @@
       <c r="E59" s="21" t="s">
         <v>261</v>
       </c>
-      <c r="F59" s="38" t="s">
+      <c r="F59" s="32" t="s">
         <v>187</v>
       </c>
       <c r="G59" s="1"/>
@@ -3717,7 +3717,7 @@
       <c r="E60" s="21" t="s">
         <v>277</v>
       </c>
-      <c r="F60" s="38" t="s">
+      <c r="F60" s="32" t="s">
         <v>195</v>
       </c>
       <c r="G60" s="1"/>
@@ -3789,7 +3789,7 @@
       <c r="E62" s="21" t="s">
         <v>261</v>
       </c>
-      <c r="F62" s="38" t="s">
+      <c r="F62" s="32" t="s">
         <v>187</v>
       </c>
       <c r="G62" s="1"/>
@@ -3829,7 +3829,7 @@
       <c r="E63" s="21" t="s">
         <v>197</v>
       </c>
-      <c r="F63" s="38" t="s">
+      <c r="F63" s="32" t="s">
         <v>198</v>
       </c>
       <c r="G63" s="1"/>
@@ -3901,7 +3901,7 @@
       <c r="E65" s="21" t="s">
         <v>261</v>
       </c>
-      <c r="F65" s="38" t="s">
+      <c r="F65" s="32" t="s">
         <v>187</v>
       </c>
       <c r="G65" s="1"/>
@@ -3941,7 +3941,7 @@
       <c r="E66" s="21" t="s">
         <v>264</v>
       </c>
-      <c r="F66" s="38" t="s">
+      <c r="F66" s="32" t="s">
         <v>201</v>
       </c>
       <c r="G66" s="1"/>
@@ -4013,7 +4013,7 @@
       <c r="E68" s="21" t="s">
         <v>261</v>
       </c>
-      <c r="F68" s="38" t="s">
+      <c r="F68" s="32" t="s">
         <v>187</v>
       </c>
       <c r="G68" s="1"/>
@@ -4053,7 +4053,7 @@
       <c r="E69" s="21" t="s">
         <v>207</v>
       </c>
-      <c r="F69" s="38" t="s">
+      <c r="F69" s="32" t="s">
         <v>208</v>
       </c>
       <c r="G69" s="1"/>
@@ -4093,7 +4093,7 @@
       <c r="E70" s="21" t="s">
         <v>212</v>
       </c>
-      <c r="F70" s="38" t="s">
+      <c r="F70" s="32" t="s">
         <v>213</v>
       </c>
       <c r="G70" s="1"/>
@@ -4133,7 +4133,7 @@
       <c r="E71" s="21" t="s">
         <v>262</v>
       </c>
-      <c r="F71" s="38" t="s">
+      <c r="F71" s="32" t="s">
         <v>40</v>
       </c>
       <c r="G71" s="1"/>
@@ -4395,7 +4395,7 @@
       <c r="E79" s="21" t="s">
         <v>224</v>
       </c>
-      <c r="F79" s="38" t="s">
+      <c r="F79" s="32" t="s">
         <v>225</v>
       </c>
       <c r="G79" s="1"/>
@@ -4435,7 +4435,7 @@
       <c r="E80" s="21" t="s">
         <v>228</v>
       </c>
-      <c r="F80" s="38" t="s">
+      <c r="F80" s="32" t="s">
         <v>229</v>
       </c>
       <c r="G80" s="1"/>
@@ -4507,7 +4507,7 @@
       <c r="E82" s="21" t="s">
         <v>224</v>
       </c>
-      <c r="F82" s="38" t="s">
+      <c r="F82" s="32" t="s">
         <v>225</v>
       </c>
       <c r="G82" s="1"/>
@@ -4547,7 +4547,7 @@
       <c r="E83" s="21" t="s">
         <v>233</v>
       </c>
-      <c r="F83" s="38" t="s">
+      <c r="F83" s="32" t="s">
         <v>234</v>
       </c>
       <c r="G83" s="1"/>
@@ -4619,7 +4619,7 @@
       <c r="E85" s="21" t="s">
         <v>224</v>
       </c>
-      <c r="F85" s="38" t="s">
+      <c r="F85" s="32" t="s">
         <v>225</v>
       </c>
       <c r="G85" s="1"/>
@@ -4659,7 +4659,7 @@
       <c r="E86" s="21" t="s">
         <v>238</v>
       </c>
-      <c r="F86" s="38" t="s">
+      <c r="F86" s="32" t="s">
         <v>239</v>
       </c>
       <c r="G86" s="1"/>
@@ -4731,7 +4731,7 @@
       <c r="E88" s="21" t="s">
         <v>224</v>
       </c>
-      <c r="F88" s="38" t="s">
+      <c r="F88" s="32" t="s">
         <v>225</v>
       </c>
       <c r="G88" s="1"/>
@@ -4771,7 +4771,7 @@
       <c r="E89" s="21" t="s">
         <v>243</v>
       </c>
-      <c r="F89" s="38" t="s">
+      <c r="F89" s="32" t="s">
         <v>244</v>
       </c>
       <c r="G89" s="1"/>
@@ -4843,7 +4843,7 @@
       <c r="E91" s="21" t="s">
         <v>224</v>
       </c>
-      <c r="F91" s="38" t="s">
+      <c r="F91" s="32" t="s">
         <v>225</v>
       </c>
       <c r="G91" s="1"/>
@@ -4883,7 +4883,7 @@
       <c r="E92" s="21" t="s">
         <v>248</v>
       </c>
-      <c r="F92" s="38" t="s">
+      <c r="F92" s="32" t="s">
         <v>249</v>
       </c>
       <c r="G92" s="1"/>
@@ -4923,7 +4923,7 @@
       <c r="E93" s="21" t="s">
         <v>251</v>
       </c>
-      <c r="F93" s="38" t="s">
+      <c r="F93" s="32" t="s">
         <v>252</v>
       </c>
       <c r="G93" s="1"/>
@@ -4995,7 +4995,7 @@
       <c r="E95" s="21" t="s">
         <v>224</v>
       </c>
-      <c r="F95" s="38" t="s">
+      <c r="F95" s="32" t="s">
         <v>225</v>
       </c>
       <c r="G95" s="1"/>
@@ -5035,7 +5035,7 @@
       <c r="E96" s="21" t="s">
         <v>256</v>
       </c>
-      <c r="F96" s="38" t="s">
+      <c r="F96" s="32" t="s">
         <v>257</v>
       </c>
       <c r="G96" s="1"/>
@@ -5075,7 +5075,7 @@
       <c r="E97" s="21" t="s">
         <v>281</v>
       </c>
-      <c r="F97" s="38" t="s">
+      <c r="F97" s="32" t="s">
         <v>260</v>
       </c>
       <c r="G97" s="1"/>
@@ -30073,16 +30073,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="33"/>
+      <c r="B1" s="44"/>
     </row>
     <row r="2" spans="1:2" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="42" t="s">
+      <c r="B2" s="36" t="s">
         <v>286</v>
       </c>
     </row>
@@ -30090,7 +30090,7 @@
       <c r="A3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="34" t="s">
         <v>10</v>
       </c>
     </row>
@@ -30110,7 +30110,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
         <v>20</v>
       </c>
@@ -30118,7 +30118,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
         <v>24</v>
       </c>
@@ -30126,7 +30126,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
         <v>29</v>
       </c>
@@ -30138,21 +30138,21 @@
       <c r="A9" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="38" t="s">
+      <c r="B9" s="32" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="34" t="s">
+      <c r="A11" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="33"/>
+      <c r="B11" s="44"/>
     </row>
     <row r="12" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B12" s="43" t="s">
+      <c r="B12" s="37" t="s">
         <v>43</v>
       </c>
     </row>
@@ -30160,7 +30160,7 @@
       <c r="A13" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="40" t="s">
+      <c r="B13" s="34" t="s">
         <v>44</v>
       </c>
     </row>
@@ -30172,7 +30172,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A15" s="8" t="s">
         <v>17</v>
       </c>
@@ -30180,7 +30180,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A16" s="8" t="s">
         <v>20</v>
       </c>
@@ -30188,7 +30188,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A17" s="8" t="s">
         <v>24</v>
       </c>
@@ -30196,7 +30196,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A18" s="8" t="s">
         <v>29</v>
       </c>
@@ -30208,21 +30208,21 @@
       <c r="A19" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B19" s="38" t="s">
+      <c r="B19" s="32" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="34" t="s">
+      <c r="A21" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="B21" s="33"/>
+      <c r="B21" s="44"/>
     </row>
     <row r="22" spans="1:6" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B22" s="42" t="s">
+      <c r="B22" s="36" t="s">
         <v>287</v>
       </c>
     </row>
@@ -30230,7 +30230,7 @@
       <c r="A23" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="40" t="s">
+      <c r="B23" s="34" t="s">
         <v>54</v>
       </c>
     </row>
@@ -30241,7 +30241,7 @@
       <c r="B24" s="21" t="s">
         <v>284</v>
       </c>
-      <c r="F24" s="41"/>
+      <c r="F24" s="35"/>
     </row>
     <row r="25" spans="1:6" ht="51" x14ac:dyDescent="0.2">
       <c r="A25" s="8" t="s">
@@ -30279,7 +30279,7 @@
       <c r="A29" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B29" s="38" t="s">
+      <c r="B29" s="32" t="s">
         <v>59</v>
       </c>
     </row>
@@ -30311,61 +30311,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
     </row>
     <row r="2" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="33"/>
+      <c r="B2" s="44"/>
       <c r="C2" s="7"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="37" t="s">
+    <row r="3" spans="1:3" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A3" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="33"/>
+      <c r="B3" s="44"/>
       <c r="C3" s="10">
         <v>46223</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="37" t="s">
+    <row r="4" spans="1:3" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A4" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="33"/>
+      <c r="B4" s="44"/>
       <c r="C4" s="9" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="102" x14ac:dyDescent="0.2">
-      <c r="A5" s="37" t="s">
+      <c r="A5" s="46" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="33"/>
-      <c r="C5" s="44" t="s">
+      <c r="B5" s="44"/>
+      <c r="C5" s="38" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="37" t="s">
+    <row r="6" spans="1:3" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A6" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="33"/>
+      <c r="B6" s="44"/>
       <c r="C6" s="9" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A7" s="37" t="s">
+      <c r="A7" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="33"/>
-      <c r="C7" s="38" t="s">
+      <c r="B7" s="44"/>
+      <c r="C7" s="32" t="s">
         <v>34</v>
       </c>
     </row>
@@ -30400,80 +30400,80 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="E1" s="36" t="s">
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="E1" s="48" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="33"/>
+      <c r="B2" s="44"/>
       <c r="C2" s="7"/>
-      <c r="E2" s="33"/>
+      <c r="E2" s="44"/>
     </row>
     <row r="3" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="37" t="s">
+      <c r="A3" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="33"/>
+      <c r="B3" s="44"/>
       <c r="C3" s="10">
         <v>46223</v>
       </c>
-      <c r="E3" s="45" t="s">
+      <c r="E3" s="51" t="s">
         <v>288</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="33"/>
+      <c r="B4" s="44"/>
       <c r="C4" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E4" s="45"/>
+      <c r="E4" s="51"/>
     </row>
     <row r="5" spans="1:5" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="47" t="s">
+      <c r="A5" s="49" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="33"/>
-      <c r="C5" s="52" t="s">
+      <c r="B5" s="44"/>
+      <c r="C5" s="42" t="s">
         <v>37</v>
       </c>
-      <c r="E5" s="45"/>
+      <c r="E5" s="51"/>
     </row>
     <row r="6" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="33"/>
-      <c r="C6" s="46" t="s">
+      <c r="B6" s="44"/>
+      <c r="C6" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="E6" s="45"/>
+      <c r="E6" s="51"/>
     </row>
     <row r="7" spans="1:5" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="47" t="s">
+      <c r="A7" s="49" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="33"/>
-      <c r="C7" s="51" t="s">
+      <c r="B7" s="44"/>
+      <c r="C7" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="E7" s="45"/>
+      <c r="E7" s="51"/>
     </row>
     <row r="8" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E8" s="45"/>
+      <c r="E8" s="51"/>
     </row>
     <row r="9" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E9" s="45"/>
+      <c r="E9" s="51"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -30509,12 +30509,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="52" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
     </row>
     <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
@@ -30534,10 +30534,10 @@
       <c r="A3" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="39" t="s">
         <v>85</v>
       </c>
-      <c r="C3" s="49" t="s">
+      <c r="C3" s="40" t="s">
         <v>86</v>
       </c>
       <c r="D3" s="9" t="s">
@@ -30548,7 +30548,7 @@
       <c r="A4" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="B4" s="46" t="s">
+      <c r="B4" s="39" t="s">
         <v>89</v>
       </c>
       <c r="C4" s="9" t="s">
@@ -30558,7 +30558,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A5" s="9" t="s">
         <v>92</v>
       </c>
@@ -30572,7 +30572,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
         <v>95</v>
       </c>
@@ -30586,7 +30586,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
         <v>96</v>
       </c>
@@ -30600,7 +30600,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
         <v>102</v>
       </c>

</xml_diff>